<commit_message>
Khôi phục nhóm Nghiên cứu & nâng cao năng lực trong hồ sơ v1.3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EV7sz8o6rnFsV7vTWvp1Kv
</commit_message>
<xml_diff>
--- a/Ho_so_khai_bao_NSLD_GPQTNB_v1.3.xlsx
+++ b/Ho_so_khai_bao_NSLD_GPQTNB_v1.3.xlsx
@@ -600,7 +600,7 @@
     <row r="2" ht="15" customHeight="1" s="21">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Phiên bản 2.1 · Theo Hướng dẫn đo lường NSLĐ TT Công nghệ nền tảng v1.0 · Đơn vị đo: ĐVCV · Bản áp dụng thử · 4 nhóm việc, 11 loại task việc</t>
+          <t>Phiên bản 2.1 · Theo Hướng dẫn đo lường NSLĐ TT Công nghệ nền tảng v1.0 · Đơn vị đo: ĐVCV · Bản áp dụng thử · 5 nhóm việc, 13 loại task việc</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>Gộp Phát triển API/Service tích hợp, Phát triển Job/Batch tính toán nghiệp vụ, Khắc phục phát hiện của đơn vị kiểm soát và Bảo trì, tối ưu, xử lý nợ kỹ thuật vào dòng Phát triển, bảo trì chức năng hệ thống. Đổi dòng Viết kịch bản và hỗ trợ kiểm thử (SIT/UAT) thành TC4D (Test Case for Dev) để làm rõ đây là việc của Developer, không phải của đội Test. Gộp Xử lý yêu cầu hỗ trợ nghiệp vụ, tra soát và đối soát; Khắc phục sự cố, khôi phục hệ thống; và Hỗ trợ vận hành, xử lý sự cố cho đơn vị ngoài thành dòng Hỗ trợ vận hành, tra soát và xử lý sự cố. Bỏ các dòng Nghiên cứu công nghệ, giải pháp mới; Đào tạo, chuẩn hóa tài liệu nội bộ; Công việc hành chính, tổng hợp số liệu. Danh mục còn 4 nhóm việc, 11 loại task việc. Các mức và ví dụ là đề xuất, cần chấm thử với team lead trước khi áp dụng chính thức.</t>
+          <t>Gộp Phát triển API/Service tích hợp, Phát triển Job/Batch tính toán nghiệp vụ, Khắc phục phát hiện của đơn vị kiểm soát và Bảo trì, tối ưu, xử lý nợ kỹ thuật vào dòng Phát triển, bảo trì chức năng hệ thống. Đổi dòng Viết kịch bản và hỗ trợ kiểm thử (SIT/UAT) thành TC4D (Test Case for Dev) để làm rõ đây là việc của Developer, không phải của đội Test. Gộp Xử lý yêu cầu hỗ trợ nghiệp vụ, tra soát và đối soát; Khắc phục sự cố, khôi phục hệ thống; và Hỗ trợ vận hành, xử lý sự cố cho đơn vị ngoài thành dòng Hỗ trợ vận hành, tra soát và xử lý sự cố. Bỏ dòng Công việc hành chính, tổng hợp số liệu. Danh mục còn 5 nhóm việc, 13 loại task việc. Các mức và ví dụ là đề xuất, cần chấm thử với team lead trước khi áp dụng chính thức.</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -2029,27 +2029,106 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1" s="21">
-      <c r="A16" s="14" t="n"/>
-      <c r="B16" s="14" t="n"/>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="14" t="n"/>
-      <c r="E16" s="16" t="n"/>
-      <c r="F16" s="14" t="n"/>
-      <c r="G16" s="16" t="n"/>
-      <c r="H16" s="14" t="n"/>
-      <c r="I16" s="14" t="n"/>
-    </row>
-    <row r="17" ht="42" customHeight="1" s="21">
-      <c r="A17" s="14" t="n"/>
-      <c r="B17" s="14" t="n"/>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="14" t="n"/>
-      <c r="E17" s="16" t="n"/>
-      <c r="F17" s="14" t="n"/>
-      <c r="G17" s="16" t="n"/>
-      <c r="H17" s="14" t="n"/>
-      <c r="I17" s="14" t="n"/>
+    <row r="16" ht="188" customHeight="1" s="21">
+      <c r="A16" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="25" t="inlineStr">
+        <is>
+          <t>Nghiên cứu &amp; nâng cao năng lực</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Nghiên cứu công nghệ, giải pháp mới</t>
+        </is>
+      </c>
+      <c r="D16" s="30" t="inlineStr">
+        <is>
+          <t>Nghiên cứu, đánh giá hoặc thực hiện POC đối với một công nghệ, sản phẩm, kiến trúc hoặc giải pháp mới chưa được lựa chọn/áp dụng chính thức; tập trung vào khả năng đáp ứng yêu cầu, ưu nhược điểm, điều kiện áp dụng và khả năng tích hợp với hệ thống hiện tại. Không áp dụng cho việc xử lý/tối ưu trực tiếp một vấn đề của hệ thống đang vận hành, được phân loại tại Task "Phát triển, bảo trì chức năng hệ thống". Đầu ra: Báo cáo/kết quả nghiên cứu, đánh giá hoặc POC và khuyến nghị áp dụng nếu có.</t>
+        </is>
+      </c>
+      <c r="E16" s="28" t="inlineStr">
+        <is>
+          <t>0,5</t>
+        </is>
+      </c>
+      <c r="F16" s="25" t="inlineStr">
+        <is>
+          <t>CTNB-22011 - Tìm hiểu production-grade, SFTP và ký số phục vụ đối soát SMS Viettel. Khảo sát ban đầu dựa trên tài liệu.</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="inlineStr">
+        <is>
+          <t>5,0</t>
+        </is>
+      </c>
+      <c r="H16" s="25" t="inlineStr">
+        <is>
+          <t>OGL-2967 - Nghiên cứu xây dựng Chatbot trên Oracle APEX. Hướng công nghệ mới, cần đánh giá nhiều phương án và có thể ảnh hưởng lựa chọn giải pháp.</t>
+        </is>
+      </c>
+      <c r="I16" s="32" t="inlineStr">
+        <is>
+          <t>Mức độ: 
+0,5 : Khảo sát nhanh trên tài liệu. 
+1 : Task cơ sở. 
+2 : So sánh nhiều phương án theo tiêu chí. 
+3 : POC chạy được trên môi trường test. 
+5 : POC cho hướng công nghệ mới, có ảnh hưởng đến lựa chọn giải pháp. 
+Lưu ý: Nếu kết quả được chuyển thành sản phẩm triển khai thực tế thì phần triển khai tính tại dòng phát triển tương ứng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="113" customHeight="1" s="21">
+      <c r="A17" s="24" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="25" t="inlineStr">
+        <is>
+          <t>Nghiên cứu &amp; nâng cao năng lực</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>Đào tạo, chuẩn hóa tài liệu nội bộ</t>
+        </is>
+      </c>
+      <c r="D17" s="30" t="inlineStr">
+        <is>
+          <t>Xây dựng hoặc chuẩn hóa tài liệu kỹ thuật/nghiệp vụ, hướng dẫn sử dụng/vận hành hoặc thực hiện một nội dung đào tạo nhằm chia sẻ và chuẩn hóa kiến thức trong nội bộ. Đầu ra: Tài liệu đào tạo/hướng dẫn/chuẩn hóa hoàn chỉnh hoặc nội dung đào tạo được thực hiện và có thể sử dụng lại.</t>
+        </is>
+      </c>
+      <c r="E17" s="28" t="inlineStr">
+        <is>
+          <t>0,5</t>
+        </is>
+      </c>
+      <c r="F17" s="25" t="inlineStr">
+        <is>
+          <t>OGL-2994 - Hướng dẫn tổng quan cấu trúc dữ liệu module ngân sách phục vụ báo cáo BI. Phạm vi nội dung hẹp.</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="inlineStr">
+        <is>
+          <t>2,0</t>
+        </is>
+      </c>
+      <c r="H17" s="25" t="inlineStr">
+        <is>
+          <t>FCRM-8884 - Tìm hiểu và hướng dẫn phân quyền báo cáo OAS cho OPN. Vừa chuẩn bị nội dung vừa hướng dẫn theo tình huống thực tế.</t>
+        </is>
+      </c>
+      <c r="I17" s="32" t="inlineStr">
+        <is>
+          <t>Mức độ: 
+0,5 : Hướng dẫn nội dung hẹp cho một người. 
+1 : Task cơ sở. 
+2 : Vừa xây dựng nội dung vừa hướng dẫn theo tình huống. 
+3 : Một bộ tài liệu chuẩn hoặc chương trình đào tạo nhiều buổi. 
+Lưu ý: Công việc quản lý đội nhóm không tính tại dòng này nếu không có đầu ra đào tạo/tài liệu độc lập.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="42" customHeight="1" s="21">
       <c r="A18" s="14" t="n"/>

</xml_diff>